<commit_message>
Sync planning SharePoint : S15
</commit_message>
<xml_diff>
--- a/Plannings 2026 S15.xlsx
+++ b/Plannings 2026 S15.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B16CE52-039B-4D77-8B5C-7A7A29AECE6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{4B16CE52-039B-4D77-8B5C-7A7A29AECE6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F953700-6C2E-4E1D-8D1C-D14D7ADDDEA7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7944,7 +7944,7 @@
       <c r="F90" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G90" s="18" t="s">
+      <c r="G90" s="54" t="s">
         <v>59</v>
       </c>
       <c r="H90" s="19"/>
@@ -7962,7 +7962,7 @@
       <c r="F91" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="G91" s="1" t="s">
+      <c r="G91" s="55" t="s">
         <v>117</v>
       </c>
       <c r="H91" s="26"/>
@@ -8843,13 +8843,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{744CE1F1-CD27-4266-9A98-F6C54EF8FFEE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A34CDE22-8465-4659-8521-E79C5228AA8B}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97F41EB0-F4AF-4816-9163-6C8ADF105326}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D1212E9-822A-401C-B398-ABE0B3D00853}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D7E64A4-E99B-45E4-820F-4A2C57506F77}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD621067-9B7A-44C8-9D5B-AA32B358918C}"/>
 </file>
</xml_diff>